<commit_message>
inter-floor time = hieght/velocity
</commit_message>
<xml_diff>
--- a/ESRA_v3/NumFloors-20-20-NumCars-5-5IncomingTraffic-30-30-InterfloorTraffic-40-40-NumSims-1.xlsx
+++ b/ESRA_v3/NumFloors-20-20-NumCars-5-5IncomingTraffic-30-30-InterfloorTraffic-40-40-NumSims-1.xlsx
@@ -434,9 +434,7 @@
           <t>Incoming_30</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>9.199999999999999</v>
-      </c>
+      <c r="B2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -456,9 +454,7 @@
           <t>Incoming_30</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>11.77777777777778</v>
-      </c>
+      <c r="B5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
both directions calculated if state==0 in car_waiting_times()
</commit_message>
<xml_diff>
--- a/ESRA_v3/NumFloors-20-20-NumCars-5-5IncomingTraffic-30-30-InterfloorTraffic-40-40-NumSims-1.xlsx
+++ b/ESRA_v3/NumFloors-20-20-NumCars-5-5IncomingTraffic-30-30-InterfloorTraffic-40-40-NumSims-1.xlsx
@@ -434,7 +434,9 @@
           <t>Incoming_30</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -454,7 +456,9 @@
           <t>Incoming_30</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>